<commit_message>
Docs: improvement round built; Range Rover reports re-exported live with the new sections
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142L4rKS2AV8rxQTDWMs7dy
</commit_message>
<xml_diff>
--- a/calculator/scripts/sw-review/rr-phev-2026-10-14/rr-phev-UK.xlsx
+++ b/calculator/scripts/sw-review/rr-phev-2026-10-14/rr-phev-UK.xlsx
@@ -16,6 +16,12 @@
     <sheet name="Vehicle map" sheetId="11" r:id="rId11"/>
     <sheet name="Schedule" sheetId="12" r:id="rId12"/>
     <sheet name="Hub rate" sheetId="13" r:id="rId13"/>
+    <sheet name="Every hub" sheetId="14" r:id="rId14"/>
+    <sheet name="Countries" sheetId="15" r:id="rId15"/>
+    <sheet name="Assumptions" sheetId="16" r:id="rId16"/>
+    <sheet name="Your figures" sheetId="17" r:id="rId17"/>
+    <sheet name="Calibration" sheetId="18" r:id="rId18"/>
+    <sheet name="Exclusions" sheetId="19" r:id="rId19"/>
   </sheets>
 </workbook>
 </file>
@@ -4005,6 +4011,2516 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I27"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>CostVision — Should-Cost Report</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>The same 52-module scope re-costed at every hub in the rate book (each at its own book rate); £M</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Hub</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Rate confidence</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Loaded £ / PM</v>
+      </c>
+      <c r="D4" t="str">
+        <v>NRE</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Lifecycle</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Total</v>
+      </c>
+      <c r="G4" t="str">
+        <v>£ / vehicle</v>
+      </c>
+      <c r="H4" t="str">
+        <v>v this costing</v>
+      </c>
+      <c r="I4" t="str">
+        <v>This costing</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Egypt</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C5">
+        <v>882.49</v>
+      </c>
+      <c r="D5">
+        <v>23.716</v>
+      </c>
+      <c r="E5">
+        <v>203.546</v>
+      </c>
+      <c r="F5">
+        <v>227.262</v>
+      </c>
+      <c r="G5">
+        <v>189.38</v>
+      </c>
+      <c r="H5">
+        <v>-76.068</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>India</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C6">
+        <v>1071.83</v>
+      </c>
+      <c r="D6">
+        <v>24.626</v>
+      </c>
+      <c r="E6">
+        <v>204.171</v>
+      </c>
+      <c r="F6">
+        <v>228.797</v>
+      </c>
+      <c r="G6">
+        <v>190.66</v>
+      </c>
+      <c r="H6">
+        <v>-74.533</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Vietnam</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C7">
+        <v>1954.56</v>
+      </c>
+      <c r="D7">
+        <v>28.868</v>
+      </c>
+      <c r="E7">
+        <v>207.084</v>
+      </c>
+      <c r="F7">
+        <v>235.952</v>
+      </c>
+      <c r="G7">
+        <v>196.63</v>
+      </c>
+      <c r="H7">
+        <v>-67.378</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Mexico</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C8">
+        <v>2100.57</v>
+      </c>
+      <c r="D8">
+        <v>29.57</v>
+      </c>
+      <c r="E8">
+        <v>207.566</v>
+      </c>
+      <c r="F8">
+        <v>237.135</v>
+      </c>
+      <c r="G8">
+        <v>197.61</v>
+      </c>
+      <c r="H8">
+        <v>-66.194</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Türkiye</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C9">
+        <v>2239.92</v>
+      </c>
+      <c r="D9">
+        <v>30.239</v>
+      </c>
+      <c r="E9">
+        <v>208.026</v>
+      </c>
+      <c r="F9">
+        <v>238.265</v>
+      </c>
+      <c r="G9">
+        <v>198.55</v>
+      </c>
+      <c r="H9">
+        <v>-65.065</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Japan</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C10">
+        <v>4051.44</v>
+      </c>
+      <c r="D10">
+        <v>38.945</v>
+      </c>
+      <c r="E10">
+        <v>214.003</v>
+      </c>
+      <c r="F10">
+        <v>252.949</v>
+      </c>
+      <c r="G10">
+        <v>210.79</v>
+      </c>
+      <c r="H10">
+        <v>-50.381</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C11">
+        <v>5198.2</v>
+      </c>
+      <c r="D11">
+        <v>44.456</v>
+      </c>
+      <c r="E11">
+        <v>217.788</v>
+      </c>
+      <c r="F11">
+        <v>262.244</v>
+      </c>
+      <c r="G11">
+        <v>218.54</v>
+      </c>
+      <c r="H11">
+        <v>-41.086</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Serbia</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C12">
+        <v>5333.46</v>
+      </c>
+      <c r="D12">
+        <v>45.106</v>
+      </c>
+      <c r="E12">
+        <v>218.234</v>
+      </c>
+      <c r="F12">
+        <v>263.34</v>
+      </c>
+      <c r="G12">
+        <v>219.45</v>
+      </c>
+      <c r="H12">
+        <v>-39.989</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Romania</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C13">
+        <v>5389.62</v>
+      </c>
+      <c r="D13">
+        <v>45.376</v>
+      </c>
+      <c r="E13">
+        <v>218.419</v>
+      </c>
+      <c r="F13">
+        <v>263.796</v>
+      </c>
+      <c r="G13">
+        <v>219.83</v>
+      </c>
+      <c r="H13">
+        <v>-39.534</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>South Korea</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C14">
+        <v>5396.03</v>
+      </c>
+      <c r="D14">
+        <v>45.407</v>
+      </c>
+      <c r="E14">
+        <v>218.44</v>
+      </c>
+      <c r="F14">
+        <v>263.848</v>
+      </c>
+      <c r="G14">
+        <v>219.87</v>
+      </c>
+      <c r="H14">
+        <v>-39.482</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>China</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C15">
+        <v>5572.77</v>
+      </c>
+      <c r="D15">
+        <v>46.256</v>
+      </c>
+      <c r="E15">
+        <v>219.024</v>
+      </c>
+      <c r="F15">
+        <v>265.28</v>
+      </c>
+      <c r="G15">
+        <v>221.07</v>
+      </c>
+      <c r="H15">
+        <v>-38.05</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Italy</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C16">
+        <v>5787.86</v>
+      </c>
+      <c r="D16">
+        <v>47.29</v>
+      </c>
+      <c r="E16">
+        <v>219.733</v>
+      </c>
+      <c r="F16">
+        <v>267.024</v>
+      </c>
+      <c r="G16">
+        <v>222.52</v>
+      </c>
+      <c r="H16">
+        <v>-36.306</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Czechia</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C17">
+        <v>6398.95</v>
+      </c>
+      <c r="D17">
+        <v>50.227</v>
+      </c>
+      <c r="E17">
+        <v>221.75</v>
+      </c>
+      <c r="F17">
+        <v>271.977</v>
+      </c>
+      <c r="G17">
+        <v>226.65</v>
+      </c>
+      <c r="H17">
+        <v>-31.353</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Hungary</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C18">
+        <v>6499.71</v>
+      </c>
+      <c r="D18">
+        <v>50.711</v>
+      </c>
+      <c r="E18">
+        <v>222.083</v>
+      </c>
+      <c r="F18">
+        <v>272.794</v>
+      </c>
+      <c r="G18">
+        <v>227.33</v>
+      </c>
+      <c r="H18">
+        <v>-30.536</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Poland</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C19">
+        <v>6823.91</v>
+      </c>
+      <c r="D19">
+        <v>52.269</v>
+      </c>
+      <c r="E19">
+        <v>223.152</v>
+      </c>
+      <c r="F19">
+        <v>275.422</v>
+      </c>
+      <c r="G19">
+        <v>229.52</v>
+      </c>
+      <c r="H19">
+        <v>-27.908</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Canada (Ontario)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C20">
+        <v>7107.59</v>
+      </c>
+      <c r="D20">
+        <v>53.633</v>
+      </c>
+      <c r="E20">
+        <v>224.088</v>
+      </c>
+      <c r="F20">
+        <v>277.721</v>
+      </c>
+      <c r="G20">
+        <v>231.43</v>
+      </c>
+      <c r="H20">
+        <v>-25.609</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>France</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C21">
+        <v>9181.28</v>
+      </c>
+      <c r="D21">
+        <v>63.598</v>
+      </c>
+      <c r="E21">
+        <v>230.932</v>
+      </c>
+      <c r="F21">
+        <v>294.53</v>
+      </c>
+      <c r="G21">
+        <v>245.44</v>
+      </c>
+      <c r="H21">
+        <v>-8.8</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Austria</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C22">
+        <v>10057.92</v>
+      </c>
+      <c r="D22">
+        <v>67.811</v>
+      </c>
+      <c r="E22">
+        <v>233.824</v>
+      </c>
+      <c r="F22">
+        <v>301.636</v>
+      </c>
+      <c r="G22">
+        <v>251.36</v>
+      </c>
+      <c r="H22">
+        <v>-1.694</v>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>United Kingdom</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C23">
+        <v>10266.91</v>
+      </c>
+      <c r="D23">
+        <v>68.816</v>
+      </c>
+      <c r="E23">
+        <v>234.514</v>
+      </c>
+      <c r="F23">
+        <v>303.33</v>
+      </c>
+      <c r="G23">
+        <v>252.77</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23" t="str">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Sweden</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C24">
+        <v>10337.91</v>
+      </c>
+      <c r="D24">
+        <v>69.157</v>
+      </c>
+      <c r="E24">
+        <v>234.748</v>
+      </c>
+      <c r="F24">
+        <v>303.905</v>
+      </c>
+      <c r="G24">
+        <v>253.25</v>
+      </c>
+      <c r="H24">
+        <v>0.576</v>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Germany</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C25">
+        <v>10605.46</v>
+      </c>
+      <c r="D25">
+        <v>70.443</v>
+      </c>
+      <c r="E25">
+        <v>235.631</v>
+      </c>
+      <c r="F25">
+        <v>306.074</v>
+      </c>
+      <c r="G25">
+        <v>255.06</v>
+      </c>
+      <c r="H25">
+        <v>2.744</v>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>USA — Michigan</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C26">
+        <v>12890.07</v>
+      </c>
+      <c r="D26">
+        <v>81.422</v>
+      </c>
+      <c r="E26">
+        <v>243.17</v>
+      </c>
+      <c r="F26">
+        <v>324.592</v>
+      </c>
+      <c r="G26">
+        <v>270.49</v>
+      </c>
+      <c r="H26">
+        <v>21.263</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>USA — California</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C27">
+        <v>19284.04</v>
+      </c>
+      <c r="D27">
+        <v>112.151</v>
+      </c>
+      <c r="E27">
+        <v>264.27</v>
+      </c>
+      <c r="F27">
+        <v>376.42</v>
+      </c>
+      <c r="G27">
+        <v>313.68</v>
+      </c>
+      <c r="H27">
+        <v>73.091</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I27"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D43"/>
+  <cols>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="80.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>CostVision — Should-Cost Report</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Every manufacturing country and the software hub it is costed at</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Country</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Software hub</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Programme total at that hub (£M)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Why this hub</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Austria</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Austria</v>
+      </c>
+      <c r="C5">
+        <v>301.636</v>
+      </c>
+      <c r="D5" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Belgium</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Germany</v>
+      </c>
+      <c r="C6">
+        <v>306.074</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Western Europe — Germany is the nearest assessed hub</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Brazil</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Mexico</v>
+      </c>
+      <c r="C7">
+        <v>237.135</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Latin America — Mexico (Guadalajara) is the assessed hub</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Bulgaria</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Romania</v>
+      </c>
+      <c r="C8">
+        <v>263.796</v>
+      </c>
+      <c r="D8" t="str">
+        <v>South-East Europe — Romania is the nearest assessed hub</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Canada (Ontario)</v>
+      </c>
+      <c r="C9">
+        <v>277.721</v>
+      </c>
+      <c r="D9" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>China</v>
+      </c>
+      <c r="B10" t="str">
+        <v>China</v>
+      </c>
+      <c r="C10">
+        <v>265.28</v>
+      </c>
+      <c r="D10" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Czech Republic</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Czechia</v>
+      </c>
+      <c r="C11">
+        <v>271.977</v>
+      </c>
+      <c r="D11" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Egypt</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Egypt</v>
+      </c>
+      <c r="C12">
+        <v>227.262</v>
+      </c>
+      <c r="D12" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>France</v>
+      </c>
+      <c r="B13" t="str">
+        <v>France</v>
+      </c>
+      <c r="C13">
+        <v>294.53</v>
+      </c>
+      <c r="D13" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Germany</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Germany</v>
+      </c>
+      <c r="C14">
+        <v>306.074</v>
+      </c>
+      <c r="D14" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Hungary</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Hungary</v>
+      </c>
+      <c r="C15">
+        <v>272.794</v>
+      </c>
+      <c r="D15" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>India</v>
+      </c>
+      <c r="B16" t="str">
+        <v>India</v>
+      </c>
+      <c r="C16">
+        <v>228.797</v>
+      </c>
+      <c r="D16" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Indonesia</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Vietnam</v>
+      </c>
+      <c r="C17">
+        <v>235.952</v>
+      </c>
+      <c r="D17" t="str">
+        <v>South-East Asia — Vietnam is the assessed hub</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Italy</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Italy</v>
+      </c>
+      <c r="C18">
+        <v>267.024</v>
+      </c>
+      <c r="D18" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Japan</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Japan</v>
+      </c>
+      <c r="C19">
+        <v>252.949</v>
+      </c>
+      <c r="D19" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Lithuania</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Poland</v>
+      </c>
+      <c r="C20">
+        <v>275.422</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Baltic — Poland is the nearest assessed hub</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Malaysia</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Vietnam</v>
+      </c>
+      <c r="C21">
+        <v>235.952</v>
+      </c>
+      <c r="D21" t="str">
+        <v>South-East Asia — Vietnam is the assessed hub</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Mexico</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Mexico</v>
+      </c>
+      <c r="C22">
+        <v>237.135</v>
+      </c>
+      <c r="D22" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Morocco</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Egypt</v>
+      </c>
+      <c r="C23">
+        <v>227.262</v>
+      </c>
+      <c r="D23" t="str">
+        <v>North Africa — Egypt (Valeo Cairo) is the assessed North-African hub</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Germany</v>
+      </c>
+      <c r="C24">
+        <v>306.074</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Western Europe — Germany is the nearest assessed hub</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Philippines</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Vietnam</v>
+      </c>
+      <c r="C25">
+        <v>235.952</v>
+      </c>
+      <c r="D25" t="str">
+        <v>South-East Asia — Vietnam is the assessed hub</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Poland</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Poland</v>
+      </c>
+      <c r="C26">
+        <v>275.422</v>
+      </c>
+      <c r="D26" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="C27">
+        <v>262.244</v>
+      </c>
+      <c r="D27" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Romania</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Romania</v>
+      </c>
+      <c r="C28">
+        <v>263.796</v>
+      </c>
+      <c r="D28" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Serbia</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Serbia</v>
+      </c>
+      <c r="C29">
+        <v>263.34</v>
+      </c>
+      <c r="D29" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Singapore</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Japan</v>
+      </c>
+      <c r="C30">
+        <v>252.949</v>
+      </c>
+      <c r="D30" t="str">
+        <v>high-cost Asian engineering — Japan is the nearest assessed hub</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Slovakia</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Czechia</v>
+      </c>
+      <c r="C31">
+        <v>271.977</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Central Europe — Czechia is the nearest assessed hub</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Slovenia</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Austria</v>
+      </c>
+      <c r="C32">
+        <v>301.636</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Central Europe — Austria is the nearest assessed hub</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>South Africa</v>
+      </c>
+      <c r="B33" t="str">
+        <v>India</v>
+      </c>
+      <c r="C33">
+        <v>228.797</v>
+      </c>
+      <c r="D33" t="str">
+        <v>no assessed African hub south of Egypt — India, the largest offshore automotive software base</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>South Korea</v>
+      </c>
+      <c r="B34" t="str">
+        <v>South Korea</v>
+      </c>
+      <c r="C34">
+        <v>263.848</v>
+      </c>
+      <c r="D34" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Spain</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="C35">
+        <v>262.244</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Iberia — the research found no Spanish embedded-automotive salary data; Portugal (Bosch Braga) is the assessed Iberian hub</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Sweden</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Sweden</v>
+      </c>
+      <c r="C36">
+        <v>303.905</v>
+      </c>
+      <c r="D36" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Taiwan</v>
+      </c>
+      <c r="B37" t="str">
+        <v>China</v>
+      </c>
+      <c r="C37">
+        <v>265.28</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Greater China — China is the assessed hub</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Thailand</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Vietnam</v>
+      </c>
+      <c r="C38">
+        <v>235.952</v>
+      </c>
+      <c r="D38" t="str">
+        <v>South-East Asia — Vietnam is the assessed hub</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Tunisia</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Egypt</v>
+      </c>
+      <c r="C39">
+        <v>227.262</v>
+      </c>
+      <c r="D39" t="str">
+        <v>North Africa — Egypt (Valeo Cairo) is the assessed North-African hub</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Turkey</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Türkiye</v>
+      </c>
+      <c r="C40">
+        <v>238.265</v>
+      </c>
+      <c r="D40" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>United Kingdom</v>
+      </c>
+      <c r="B41" t="str">
+        <v>United Kingdom</v>
+      </c>
+      <c r="C41">
+        <v>303.33</v>
+      </c>
+      <c r="D41" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>United States</v>
+      </c>
+      <c r="B42" t="str">
+        <v>USA — Michigan</v>
+      </c>
+      <c r="C42">
+        <v>324.592</v>
+      </c>
+      <c r="D42" t="str">
+        <v>United States — Michigan (Detroit / Ann Arbor OEM software centres); choose California for Bay Area teams</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Vietnam</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Vietnam</v>
+      </c>
+      <c r="C43">
+        <v>235.952</v>
+      </c>
+      <c r="D43" t="str">
+        <v>its own assessed hub</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D43"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B15"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="120.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>CostVision — Should-Cost Report</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Assumption</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Basis</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Connected service per vehicle</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Each connected vehicle served 8 years from build — the median of current OEM terms: GM OnStar Basics 8 yr (MY2025+), Tesla Standard Connectivity 8 yr (ordered after 20 Jul 2022), Toyota up to 10 yr, Mercedes-Benz mbrace Connect 5 yr (US); OEM pages, re-checked 14 Oct 2026. A 2G / 3G / 4G shutdown can end it sooner.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Map-data subscription</v>
+      </c>
+      <c r="B5" t="str">
+        <v>3 years of map updates per vehicle — Nissan, Subaru, Hyundai, Honda (2021–24) include 3; some brands 5 or lifetime (OEM pages, read from search results).</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Cloud £ per connected vehicle-year</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Module cloud £ / yr ÷ reference fleet — an unsourced estimate (≈ £10.8 per connected vehicle-year with every module in scope). No OEM publishes a back-end cost; the only list price, AWS IoT FleetWise (US$0.60 / 0.45 per vehicle-month, messages and storage extra; closed to new customers 30 Apr 2026), is US$5.4–7.2 per vehicle-year for data collection alone.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Development window</v>
+      </c>
+      <c r="B7" t="str">
+        <v>54 months feasibility → SOP: Volkswagen's stated development cycle (IAA 2023; target 36 months). GM "around four years" (2022); Chinese OEMs ~18–24 months. Set your programme's own.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Development tools</v>
+      </c>
+      <c r="B8" t="str">
+        <v>CostVision estimate £39,500 per engineer-seat-year — the module catalogue's tool £ at the default programme ÷ its engineer-years; no public seat price (Vector CANoe is quote-only).</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Maintenance profile</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Module % of development + verification + integration a year: in full for 3 years after SOP, then 50 % — rule of thumb (15–25 % a year, Edana; 21–26 % median years 1–3, 24 DACH SaaS products), not automotive-measured.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Security support after the last build</v>
+      </c>
+      <c r="B10" t="str">
+        <v>After the last build: each module's tail sustaining team × 25 % for 10 years — the duty is regulatory (UN R155: the post-production phase runs "until the end-of-life of all vehicles under the vehicle type"; R156: updates over the vehicles' lifetime); 10 years = Volkswagen / CARIAD's stated software support after end of production (2023, via the press); 25 % is a CostVision assumption — no published cost.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Homologation</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Type approval ≈ $1M (S&amp;P Global: R155 on one legacy model "can easily exceed $1M"); ISO 26262 assessor £600k (ASIL-D) / £250k; organisation CSMS £1.5M + SUMS £0.8M ÷ vehicle types sharing them — CostVision estimates.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Supplier margin (bought development)</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Each column re-costs the scope with that development source. A supplier's price = its effort factor ÷ (1 − 11.7 % margin), so buying is cheaper only if the supplier needs ≤ 88.3 % of the in-house effort (reuse, a cheaper hub mix).</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Effort catalogue (person-months per module)</v>
+      </c>
+      <c r="B13" t="str">
+        <v>CostVision catalogue — no published automotive productivity source was found (the defence data in Clark &amp; Madachy's cost-estimation manual is the next source to read). Calibrate on your own actuals or size modules in KSLOC.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Reuse, complexity factors</v>
+      </c>
+      <c r="B14" t="str">
+        <v>CostVision catalogue factors — no published source.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>ASIL factor</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Solcept engineering blog (× 1.4 to ASIL-B, × 1.3 B → D); A and C interpolated — Low confidence.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C5"/>
+  <cols>
+    <col min="1" max="1" width="50.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>CostVision — Should-Cost Report</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Figures you entered — they replace catalogue figures and are graded "your figures"</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Line</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Value as entered (inputs are in GBP)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Source</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>none entered yet</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E56"/>
+  <cols>
+    <col min="1" max="1" width="44.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>CostVision — Should-Cost Report</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Uncalibrated — log what these modules actually took, largest first</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Module</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Person-months</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Engineering (£M)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Share (%)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Cumulative (%)</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Camera Perception Stack</v>
+      </c>
+      <c r="B5">
+        <v>303.8</v>
+      </c>
+      <c r="C5">
+        <v>3.119</v>
+      </c>
+      <c r="D5">
+        <v>6.32</v>
+      </c>
+      <c r="E5">
+        <v>6.32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>IVI Operating System (Android Automotive / QNX)</v>
+      </c>
+      <c r="B6">
+        <v>248.4</v>
+      </c>
+      <c r="C6">
+        <v>2.551</v>
+      </c>
+      <c r="D6">
+        <v>5.17</v>
+      </c>
+      <c r="E6">
+        <v>11.49</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Sensor Fusion Engine</v>
+      </c>
+      <c r="B7">
+        <v>245.6</v>
+      </c>
+      <c r="C7">
+        <v>2.521</v>
+      </c>
+      <c r="D7">
+        <v>5.11</v>
+      </c>
+      <c r="E7">
+        <v>16.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>BMS Core Software</v>
+      </c>
+      <c r="B8">
+        <v>211</v>
+      </c>
+      <c r="C8">
+        <v>2.167</v>
+      </c>
+      <c r="D8">
+        <v>4.39</v>
+      </c>
+      <c r="E8">
+        <v>20.99</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Vehicle Motion Management (VMM)</v>
+      </c>
+      <c r="B9">
+        <v>210.2</v>
+      </c>
+      <c r="C9">
+        <v>2.159</v>
+      </c>
+      <c r="D9">
+        <v>4.37</v>
+      </c>
+      <c r="E9">
+        <v>25.37</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Hybrid Supervisory Control &amp; Energy Management</v>
+      </c>
+      <c r="B10">
+        <v>210.2</v>
+      </c>
+      <c r="C10">
+        <v>2.159</v>
+      </c>
+      <c r="D10">
+        <v>4.37</v>
+      </c>
+      <c r="E10">
+        <v>29.74</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Path Planning Algorithms</v>
+      </c>
+      <c r="B11">
+        <v>202.2</v>
+      </c>
+      <c r="C11">
+        <v>2.076</v>
+      </c>
+      <c r="D11">
+        <v>4.21</v>
+      </c>
+      <c r="E11">
+        <v>33.95</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Highway Assist / Traffic Jam Assist</v>
+      </c>
+      <c r="B12">
+        <v>196</v>
+      </c>
+      <c r="C12">
+        <v>2.013</v>
+      </c>
+      <c r="D12">
+        <v>4.08</v>
+      </c>
+      <c r="E12">
+        <v>38.03</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>EDU (Electric Drive Unit) Control Software</v>
+      </c>
+      <c r="B13">
+        <v>159.2</v>
+      </c>
+      <c r="C13">
+        <v>1.634</v>
+      </c>
+      <c r="D13">
+        <v>3.31</v>
+      </c>
+      <c r="E13">
+        <v>41.34</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Control Algorithms (ACC / LKA / AEB)</v>
+      </c>
+      <c r="B14">
+        <v>152.4</v>
+      </c>
+      <c r="C14">
+        <v>1.565</v>
+      </c>
+      <c r="D14">
+        <v>3.17</v>
+      </c>
+      <c r="E14">
+        <v>44.51</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Engine Management Software (ECU)</v>
+      </c>
+      <c r="B15">
+        <v>150.3</v>
+      </c>
+      <c r="C15">
+        <v>1.543</v>
+      </c>
+      <c r="D15">
+        <v>3.13</v>
+      </c>
+      <c r="E15">
+        <v>47.64</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Zonal Architecture Software</v>
+      </c>
+      <c r="B16">
+        <v>144.6</v>
+      </c>
+      <c r="C16">
+        <v>1.484</v>
+      </c>
+      <c r="D16">
+        <v>3.01</v>
+      </c>
+      <c r="E16">
+        <v>50.65</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Radar Processing Stack</v>
+      </c>
+      <c r="B17">
+        <v>127.4</v>
+      </c>
+      <c r="C17">
+        <v>1.308</v>
+      </c>
+      <c r="D17">
+        <v>2.65</v>
+      </c>
+      <c r="E17">
+        <v>53.3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Inverter Control Algorithms</v>
+      </c>
+      <c r="B18">
+        <v>125</v>
+      </c>
+      <c r="C18">
+        <v>1.283</v>
+      </c>
+      <c r="D18">
+        <v>2.6</v>
+      </c>
+      <c r="E18">
+        <v>55.9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Driver Monitoring Software (DMS)</v>
+      </c>
+      <c r="B19">
+        <v>120.9</v>
+      </c>
+      <c r="C19">
+        <v>1.242</v>
+      </c>
+      <c r="D19">
+        <v>2.52</v>
+      </c>
+      <c r="E19">
+        <v>58.41</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Chassis Control Software</v>
+      </c>
+      <c r="B20">
+        <v>118.2</v>
+      </c>
+      <c r="C20">
+        <v>1.213</v>
+      </c>
+      <c r="D20">
+        <v>2.46</v>
+      </c>
+      <c r="E20">
+        <v>60.87</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Motor Control (FOC/DTC/SVPWM)</v>
+      </c>
+      <c r="B21">
+        <v>118</v>
+      </c>
+      <c r="C21">
+        <v>1.212</v>
+      </c>
+      <c r="D21">
+        <v>2.46</v>
+      </c>
+      <c r="E21">
+        <v>63.33</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>App Framework &amp; HMI Layer</v>
+      </c>
+      <c r="B22">
+        <v>112.1</v>
+      </c>
+      <c r="C22">
+        <v>1.151</v>
+      </c>
+      <c r="D22">
+        <v>2.33</v>
+      </c>
+      <c r="E22">
+        <v>65.66</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Predictive Active Suspension &amp; Body Control</v>
+      </c>
+      <c r="B23">
+        <v>108.6</v>
+      </c>
+      <c r="C23">
+        <v>1.115</v>
+      </c>
+      <c r="D23">
+        <v>2.26</v>
+      </c>
+      <c r="E23">
+        <v>67.92</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>AUTOSAR Adaptive Platform</v>
+      </c>
+      <c r="B24">
+        <v>104.6</v>
+      </c>
+      <c r="C24">
+        <v>1.074</v>
+      </c>
+      <c r="D24">
+        <v>2.18</v>
+      </c>
+      <c r="E24">
+        <v>70.1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Transmission Control Software (TCU)</v>
+      </c>
+      <c r="B25">
+        <v>103.4</v>
+      </c>
+      <c r="C25">
+        <v>1.062</v>
+      </c>
+      <c r="D25">
+        <v>2.15</v>
+      </c>
+      <c r="E25">
+        <v>72.25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Vehicle Voice Assistant</v>
+      </c>
+      <c r="B26">
+        <v>99.8</v>
+      </c>
+      <c r="C26">
+        <v>1.024</v>
+      </c>
+      <c r="D26">
+        <v>2.08</v>
+      </c>
+      <c r="E26">
+        <v>74.33</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Cloud Backend Services</v>
+      </c>
+      <c r="B27">
+        <v>96.3</v>
+      </c>
+      <c r="C27">
+        <v>0.988</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27">
+        <v>76.33</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>AUTOSAR Classic BSW &amp; Integration</v>
+      </c>
+      <c r="B28">
+        <v>81.9</v>
+      </c>
+      <c r="C28">
+        <v>0.841</v>
+      </c>
+      <c r="D28">
+        <v>1.7</v>
+      </c>
+      <c r="E28">
+        <v>78.03</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>SOC/SOH/SOE Estimation Models</v>
+      </c>
+      <c r="B29">
+        <v>80.8</v>
+      </c>
+      <c r="C29">
+        <v>0.83</v>
+      </c>
+      <c r="D29">
+        <v>1.68</v>
+      </c>
+      <c r="E29">
+        <v>79.72</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Automated Parking &amp; Surround-View</v>
+      </c>
+      <c r="B30">
+        <v>80.8</v>
+      </c>
+      <c r="C30">
+        <v>0.83</v>
+      </c>
+      <c r="D30">
+        <v>1.68</v>
+      </c>
+      <c r="E30">
+        <v>81.4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Body Control Software</v>
+      </c>
+      <c r="B31">
+        <v>57.5</v>
+      </c>
+      <c r="C31">
+        <v>0.59</v>
+      </c>
+      <c r="D31">
+        <v>1.2</v>
+      </c>
+      <c r="E31">
+        <v>82.59</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>OTA Update Manager (Vehicle-side)</v>
+      </c>
+      <c r="B32">
+        <v>52.3</v>
+      </c>
+      <c r="C32">
+        <v>0.537</v>
+      </c>
+      <c r="D32">
+        <v>1.09</v>
+      </c>
+      <c r="E32">
+        <v>83.68</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Telematics Control Unit (TCU) Software</v>
+      </c>
+      <c r="B33">
+        <v>51.4</v>
+      </c>
+      <c r="C33">
+        <v>0.528</v>
+      </c>
+      <c r="D33">
+        <v>1.07</v>
+      </c>
+      <c r="E33">
+        <v>84.75</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Battery Thermal Management Software</v>
+      </c>
+      <c r="B34">
+        <v>48.1</v>
+      </c>
+      <c r="C34">
+        <v>0.494</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34">
+        <v>85.75</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Gateway ECU Software</v>
+      </c>
+      <c r="B35">
+        <v>47.4</v>
+      </c>
+      <c r="C35">
+        <v>0.487</v>
+      </c>
+      <c r="D35">
+        <v>0.99</v>
+      </c>
+      <c r="E35">
+        <v>86.74</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Navigation Stack</v>
+      </c>
+      <c r="B36">
+        <v>43.9</v>
+      </c>
+      <c r="C36">
+        <v>0.451</v>
+      </c>
+      <c r="D36">
+        <v>0.91</v>
+      </c>
+      <c r="E36">
+        <v>87.65</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Fast-Charging Control Software</v>
+      </c>
+      <c r="B37">
+        <v>40.8</v>
+      </c>
+      <c r="C37">
+        <v>0.419</v>
+      </c>
+      <c r="D37">
+        <v>0.85</v>
+      </c>
+      <c r="E37">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>AR Head-Up Display &amp; AR Navigation</v>
+      </c>
+      <c r="B38">
+        <v>39.5</v>
+      </c>
+      <c r="C38">
+        <v>0.406</v>
+      </c>
+      <c r="D38">
+        <v>0.82</v>
+      </c>
+      <c r="E38">
+        <v>89.32</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Premium Audio DSP &amp; Active Noise Control</v>
+      </c>
+      <c r="B39">
+        <v>38.2</v>
+      </c>
+      <c r="C39">
+        <v>0.392</v>
+      </c>
+      <c r="D39">
+        <v>0.79</v>
+      </c>
+      <c r="E39">
+        <v>90.12</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Regenerative Braking Software</v>
+      </c>
+      <c r="B40">
+        <v>37.6</v>
+      </c>
+      <c r="C40">
+        <v>0.386</v>
+      </c>
+      <c r="D40">
+        <v>0.78</v>
+      </c>
+      <c r="E40">
+        <v>90.9</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Cell Balancing Algorithms</v>
+      </c>
+      <c r="B41">
+        <v>36.6</v>
+      </c>
+      <c r="C41">
+        <v>0.376</v>
+      </c>
+      <c r="D41">
+        <v>0.76</v>
+      </c>
+      <c r="E41">
+        <v>91.66</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Secure Boot &amp; Root of Trust</v>
+      </c>
+      <c r="B42">
+        <v>35.9</v>
+      </c>
+      <c r="C42">
+        <v>0.368</v>
+      </c>
+      <c r="D42">
+        <v>0.75</v>
+      </c>
+      <c r="E42">
+        <v>92.41</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Secure OTA Software Update Framework</v>
+      </c>
+      <c r="B43">
+        <v>35.3</v>
+      </c>
+      <c r="C43">
+        <v>0.362</v>
+      </c>
+      <c r="D43">
+        <v>0.73</v>
+      </c>
+      <c r="E43">
+        <v>93.14</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Intrusion Detection System (IDS)</v>
+      </c>
+      <c r="B44">
+        <v>35.1</v>
+      </c>
+      <c r="C44">
+        <v>0.36</v>
+      </c>
+      <c r="D44">
+        <v>0.73</v>
+      </c>
+      <c r="E44">
+        <v>93.87</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Emissions After-treatment &amp; OBD</v>
+      </c>
+      <c r="B45">
+        <v>34.4</v>
+      </c>
+      <c r="C45">
+        <v>0.353</v>
+      </c>
+      <c r="D45">
+        <v>0.71</v>
+      </c>
+      <c r="E45">
+        <v>94.59</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Bluetooth / WiFi / 5G Connectivity Stack</v>
+      </c>
+      <c r="B46">
+        <v>34.1</v>
+      </c>
+      <c r="C46">
+        <v>0.351</v>
+      </c>
+      <c r="D46">
+        <v>0.71</v>
+      </c>
+      <c r="E46">
+        <v>95.3</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Data Pipeline &amp; Telemetry</v>
+      </c>
+      <c r="B47">
+        <v>33.9</v>
+      </c>
+      <c r="C47">
+        <v>0.348</v>
+      </c>
+      <c r="D47">
+        <v>0.71</v>
+      </c>
+      <c r="E47">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Climate &amp; Thermal Comfort Control</v>
+      </c>
+      <c r="B48">
+        <v>27.6</v>
+      </c>
+      <c r="C48">
+        <v>0.283</v>
+      </c>
+      <c r="D48">
+        <v>0.57</v>
+      </c>
+      <c r="E48">
+        <v>96.58</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Diagnostics (UDS / OBD-II)</v>
+      </c>
+      <c r="B49">
+        <v>26.4</v>
+      </c>
+      <c r="C49">
+        <v>0.271</v>
+      </c>
+      <c r="D49">
+        <v>0.55</v>
+      </c>
+      <c r="E49">
+        <v>97.13</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Key Management System</v>
+      </c>
+      <c r="B50">
+        <v>25.9</v>
+      </c>
+      <c r="C50">
+        <v>0.265</v>
+      </c>
+      <c r="D50">
+        <v>0.54</v>
+      </c>
+      <c r="E50">
+        <v>97.66</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>CAN / LIN / FlexRay / Ethernet Communication Stacks</v>
+      </c>
+      <c r="B51">
+        <v>24.7</v>
+      </c>
+      <c r="C51">
+        <v>0.254</v>
+      </c>
+      <c r="D51">
+        <v>0.51</v>
+      </c>
+      <c r="E51">
+        <v>98.18</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Encryption Modules &amp; Crypto Stack</v>
+      </c>
+      <c r="B52">
+        <v>21</v>
+      </c>
+      <c r="C52">
+        <v>0.216</v>
+      </c>
+      <c r="D52">
+        <v>0.44</v>
+      </c>
+      <c r="E52">
+        <v>98.62</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Ultrasonic Processing Software</v>
+      </c>
+      <c r="B53">
+        <v>19.3</v>
+      </c>
+      <c r="C53">
+        <v>0.198</v>
+      </c>
+      <c r="D53">
+        <v>0.4</v>
+      </c>
+      <c r="E53">
+        <v>99.02</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>RTOS &amp; OS Porting</v>
+      </c>
+      <c r="B54">
+        <v>17.5</v>
+      </c>
+      <c r="C54">
+        <v>0.18</v>
+      </c>
+      <c r="D54">
+        <v>0.36</v>
+      </c>
+      <c r="E54">
+        <v>99.38</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Fleet Management &amp; Analytics Software</v>
+      </c>
+      <c r="B55">
+        <v>17.2</v>
+      </c>
+      <c r="C55">
+        <v>0.176</v>
+      </c>
+      <c r="D55">
+        <v>0.36</v>
+      </c>
+      <c r="E55">
+        <v>99.74</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Time Synchronisation &amp; Network Management</v>
+      </c>
+      <c r="B56">
+        <v>12.6</v>
+      </c>
+      <c r="C56">
+        <v>0.129</v>
+      </c>
+      <c r="D56">
+        <v>0.26</v>
+      </c>
+      <c r="E56">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E56"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C14"/>
+  <cols>
+    <col min="1" max="1" width="50.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>CostVision — Should-Cost Report</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Catalogue modules not in this programme</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Module</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Domain</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Why not</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Digital Key (UWB/BLE) &amp; Secure Access</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Infotainment, Connectivity &amp; UX</v>
+      </c>
+      <c r="C5" t="str">
+        <v>not confirmed for this vehicle — excluded rather than assumed</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>48 V Belt Starter-Generator &amp; Battery Control</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Powertrain &amp; Battery</v>
+      </c>
+      <c r="C6" t="str">
+        <v>a 48 V mild-hybrid starter-generator; not this drivetrain</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Vehicle software the catalogue has no module for (review judgement) — not in the total unless added as your module</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Occupant restraint (airbag) control</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>On-board AC charger and DC-DC converter control (the charging module covers DC fast-charge protocols)</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Electric power steering and electric parking brake base software</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Tyre-pressure monitoring</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Seat memory / massage and other comfort ECUs beyond climate and body control</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Trailer functions</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C13"/>

</xml_diff>